<commit_message>
Fix element navigation target for screen-auth in EmergencyPage and AuthPage
</commit_message>
<xml_diff>
--- a/testing/selenium-web/reports/excel/E2E_Report.xlsx
+++ b/testing/selenium-web/reports/excel/E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="52">
   <si>
     <t>Metric</t>
   </si>
@@ -25,7 +25,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>5/8/2026, 8:24:12 pm</t>
+    <t>6/8/2026, 10:40:54 am</t>
   </si>
   <si>
     <t>Environment</t>
@@ -55,7 +55,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>23 ms</t>
+    <t>12145 ms</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -82,13 +82,13 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>TC-1</t>
-  </si>
-  <si>
-    <t>Web Module</t>
-  </si>
-  <si>
-    <t>Initial Test</t>
+    <t>WEB-AUTH-1785993052517</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t>WEB-AUTH-01: Should display authentication form with empty field validation</t>
   </si>
   <si>
     <t>Chrome</t>
@@ -97,13 +97,34 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-08-05T14:54:12.769Z</t>
-  </si>
-  <si>
-    <t>2026-08-05T14:54:12.790Z</t>
-  </si>
-  <si>
-    <t>10ms</t>
+    <t>2026-08-06T05:10:52.518Z</t>
+  </si>
+  <si>
+    <t>972ms</t>
+  </si>
+  <si>
+    <t>WEB-AUTH-1785993053666</t>
+  </si>
+  <si>
+    <t>WEB-AUTH-02: Should validate invalid email string input</t>
+  </si>
+  <si>
+    <t>2026-08-06T05:10:53.666Z</t>
+  </si>
+  <si>
+    <t>1147ms</t>
+  </si>
+  <si>
+    <t>WEB-AUTH-1785993054589</t>
+  </si>
+  <si>
+    <t>WEB-AUTH-03: Should sign in successfully with valid user credentials</t>
+  </si>
+  <si>
+    <t>2026-08-06T05:10:54.589Z</t>
+  </si>
+  <si>
+    <t>922ms</t>
   </si>
   <si>
     <t>Test Name</t>
@@ -128,6 +149,27 @@
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>2026-08-06T05:10:52.515Z</t>
+  </si>
+  <si>
+    <t>Submitted empty email &amp; password</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-08-06T05:10:53.665Z</t>
+  </si>
+  <si>
+    <t>Checked email format validation rule</t>
+  </si>
+  <si>
+    <t>2026-08-06T05:10:54.588Z</t>
+  </si>
+  <si>
+    <t>User authenticated cleanly</t>
   </si>
 </sst>
 </file>
@@ -550,7 +592,7 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -558,7 +600,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -601,7 +643,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -659,10 +701,62 @@
         <v>27</v>
       </c>
       <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
         <v>28</v>
       </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -685,19 +779,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -708,7 +802,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -720,19 +814,70 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>37</v>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>